<commit_message>
Base de turnover atualizada automaticamente (14/09/2026 10:01)
</commit_message>
<xml_diff>
--- a/data/dados.xlsx
+++ b/data/dados.xlsx
@@ -34219,13 +34219,19 @@
       <c r="B935" s="3" t="n">
         <v>46223</v>
       </c>
-      <c r="C935" s="3" t="n"/>
+      <c r="C935" s="3" t="n">
+        <v>46272</v>
+      </c>
       <c r="D935" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E935" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E935" s="2" t="inlineStr">
+        <is>
+          <t>04-DISPENSA COM JUSTA CAUSA</t>
+        </is>
+      </c>
       <c r="F935" s="2" t="inlineStr">
         <is>
           <t>ASSISTENTE DE ALIMENTOS E BEBIDAS JUNIOR</t>

</xml_diff>

<commit_message>
Base de turnover atualizada automaticamente (17/09/2026 10:01)
</commit_message>
<xml_diff>
--- a/data/dados.xlsx
+++ b/data/dados.xlsx
@@ -35899,13 +35899,19 @@
       <c r="B982" s="3" t="n">
         <v>46160</v>
       </c>
-      <c r="C982" s="3" t="n"/>
+      <c r="C982" s="3" t="n">
+        <v>46276</v>
+      </c>
       <c r="D982" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E982" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E982" s="2" t="inlineStr">
+        <is>
+          <t>07-ABANDONO DE EMPREGO</t>
+        </is>
+      </c>
       <c r="F982" s="2" t="inlineStr">
         <is>
           <t>ATENDENTE DE SALAO JUNIOR</t>
@@ -38365,46 +38371,52 @@
     <row r="1051">
       <c r="A1051" s="2" t="inlineStr">
         <is>
-          <t>NATANAEL PRADO FRANCISCO</t>
+          <t>NATHALIA KRISHINA GIARDINO MOURA</t>
         </is>
       </c>
       <c r="B1051" s="3" t="n">
-        <v>45810</v>
-      </c>
-      <c r="C1051" s="3" t="n"/>
+        <v>45323</v>
+      </c>
+      <c r="C1051" s="3" t="n">
+        <v>45474</v>
+      </c>
       <c r="D1051" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E1051" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E1051" s="2" t="inlineStr">
+        <is>
+          <t>06-PEDIDO DE DEMISSÃO</t>
+        </is>
+      </c>
       <c r="F1051" s="2" t="inlineStr">
         <is>
-          <t>ATENDENTE DE SALAO JUNIOR</t>
+          <t>ASSISTENTE DE ALIMENTOS E BEBIDAS JUNIOR</t>
         </is>
       </c>
       <c r="G1051" s="2" t="inlineStr">
         <is>
-          <t>SALÃO</t>
+          <t>COZINHA</t>
         </is>
       </c>
       <c r="H1051" s="2" t="inlineStr">
         <is>
-          <t>13-CABANA CAMPINAS</t>
+          <t>19-CABANA CAMPO BELO</t>
         </is>
       </c>
     </row>
     <row r="1052">
       <c r="A1052" s="2" t="inlineStr">
         <is>
-          <t>NATHALIA KRISHINA GIARDINO MOURA</t>
+          <t>NATHALIA LOURENCO LEDO</t>
         </is>
       </c>
       <c r="B1052" s="3" t="n">
-        <v>45323</v>
+        <v>45425</v>
       </c>
       <c r="C1052" s="3" t="n">
-        <v>45474</v>
+        <v>46236</v>
       </c>
       <c r="D1052" s="4" t="inlineStr">
         <is>
@@ -38418,125 +38430,119 @@
       </c>
       <c r="F1052" s="2" t="inlineStr">
         <is>
-          <t>ASSISTENTE DE ALIMENTOS E BEBIDAS JUNIOR</t>
+          <t>ANALISTA DE EXPERIENCIA DO CONSUMIDOR JUNIOR</t>
         </is>
       </c>
       <c r="G1052" s="2" t="inlineStr">
         <is>
-          <t>COZINHA</t>
+          <t>OPERAÇÕES LOJAS</t>
         </is>
       </c>
       <c r="H1052" s="2" t="inlineStr">
         <is>
-          <t>19-CABANA CAMPO BELO</t>
+          <t>01-CABANA MATRIZ</t>
         </is>
       </c>
     </row>
     <row r="1053">
       <c r="A1053" s="2" t="inlineStr">
         <is>
-          <t>NATHALIA LOURENCO LEDO</t>
+          <t>NATHALIA NEVES CHAVES</t>
         </is>
       </c>
       <c r="B1053" s="3" t="n">
-        <v>45425</v>
-      </c>
-      <c r="C1053" s="3" t="n">
-        <v>46236</v>
-      </c>
+        <v>46055</v>
+      </c>
+      <c r="C1053" s="3" t="n"/>
       <c r="D1053" s="4" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="E1053" s="2" t="inlineStr">
-        <is>
-          <t>06-PEDIDO DE DEMISSÃO</t>
-        </is>
-      </c>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E1053" s="2" t="n"/>
       <c r="F1053" s="2" t="inlineStr">
         <is>
-          <t>ANALISTA DE EXPERIENCIA DO CONSUMIDOR JUNIOR</t>
+          <t>ATENDENTE DE SALAO JUNIOR</t>
         </is>
       </c>
       <c r="G1053" s="2" t="inlineStr">
         <is>
-          <t>OPERAÇÕES LOJAS</t>
+          <t>SALÃO</t>
         </is>
       </c>
       <c r="H1053" s="2" t="inlineStr">
         <is>
-          <t>01-CABANA MATRIZ</t>
+          <t>11-CABANA ALPHAVILLE</t>
         </is>
       </c>
     </row>
     <row r="1054">
       <c r="A1054" s="2" t="inlineStr">
         <is>
-          <t>NATHALIA NEVES CHAVES</t>
+          <t>NATHALIA SANTOS AGUIAR</t>
         </is>
       </c>
       <c r="B1054" s="3" t="n">
-        <v>46055</v>
-      </c>
-      <c r="C1054" s="3" t="n"/>
+        <v>45784</v>
+      </c>
+      <c r="C1054" s="3" t="n">
+        <v>45792</v>
+      </c>
       <c r="D1054" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E1054" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E1054" s="2" t="inlineStr">
+        <is>
+          <t>14-PEDIDO ANTES TERMINO CONTRATO</t>
+        </is>
+      </c>
       <c r="F1054" s="2" t="inlineStr">
         <is>
-          <t>ATENDENTE DE SALAO JUNIOR</t>
+          <t>COORDENADOR DE SALAO</t>
         </is>
       </c>
       <c r="G1054" s="2" t="inlineStr">
         <is>
-          <t>SALÃO</t>
+          <t>LIDERANÇA LOJA</t>
         </is>
       </c>
       <c r="H1054" s="2" t="inlineStr">
         <is>
-          <t>11-CABANA ALPHAVILLE</t>
+          <t>32-CABANA TATUAPE</t>
         </is>
       </c>
     </row>
     <row r="1055">
       <c r="A1055" s="2" t="inlineStr">
         <is>
-          <t>NATHALIA SANTOS AGUIAR</t>
+          <t>NATHALY PRADO FRANCISCO</t>
         </is>
       </c>
       <c r="B1055" s="3" t="n">
-        <v>45784</v>
-      </c>
-      <c r="C1055" s="3" t="n">
-        <v>45792</v>
-      </c>
+        <v>45810</v>
+      </c>
+      <c r="C1055" s="3" t="n"/>
       <c r="D1055" s="4" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="E1055" s="2" t="inlineStr">
-        <is>
-          <t>14-PEDIDO ANTES TERMINO CONTRATO</t>
-        </is>
-      </c>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E1055" s="2" t="n"/>
       <c r="F1055" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE SALAO</t>
+          <t>ATENDENTE DE SALAO JUNIOR</t>
         </is>
       </c>
       <c r="G1055" s="2" t="inlineStr">
         <is>
-          <t>LIDERANÇA LOJA</t>
+          <t>SALÃO</t>
         </is>
       </c>
       <c r="H1055" s="2" t="inlineStr">
         <is>
-          <t>32-CABANA TATUAPE</t>
+          <t>13-CABANA CAMPINAS</t>
         </is>
       </c>
     </row>
@@ -39651,13 +39657,19 @@
       <c r="B1087" s="3" t="n">
         <v>45852</v>
       </c>
-      <c r="C1087" s="3" t="n"/>
+      <c r="C1087" s="3" t="n">
+        <v>46276</v>
+      </c>
       <c r="D1087" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E1087" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E1087" s="2" t="inlineStr">
+        <is>
+          <t>01-DISPENSA SEM JUSTA CAUSA AVISO INDENIZADO</t>
+        </is>
+      </c>
       <c r="F1087" s="2" t="inlineStr">
         <is>
           <t>ATENDENTE DE SALAO JUNIOR</t>

</xml_diff>

<commit_message>
Base de turnover atualizada automaticamente (29/09/2026 10:01)
</commit_message>
<xml_diff>
--- a/data/dados.xlsx
+++ b/data/dados.xlsx
@@ -2135,13 +2135,19 @@
       <c r="B47" s="3" t="n">
         <v>46254</v>
       </c>
-      <c r="C47" s="3" t="n"/>
+      <c r="C47" s="3" t="n">
+        <v>46286</v>
+      </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>14-PEDIDO ANTES TERMINO CONTRATO</t>
+        </is>
+      </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
           <t>ATENDENTE DE SALAO JUNIOR</t>
@@ -9001,13 +9007,19 @@
       <c r="B238" s="3" t="n">
         <v>46251</v>
       </c>
-      <c r="C238" s="3" t="n"/>
+      <c r="C238" s="3" t="n">
+        <v>46287</v>
+      </c>
       <c r="D238" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E238" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="inlineStr">
+        <is>
+          <t>03-DISPENSA ANTES TERMINO CONTRATO</t>
+        </is>
+      </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
           <t>ASSISTENTE DE ALIMENTOS E BEBIDAS JUNIOR</t>
@@ -10839,13 +10851,19 @@
       <c r="B289" s="3" t="n">
         <v>46244</v>
       </c>
-      <c r="C289" s="3" t="n"/>
+      <c r="C289" s="3" t="n">
+        <v>46287</v>
+      </c>
       <c r="D289" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E289" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E289" s="2" t="inlineStr">
+        <is>
+          <t>04-DISPENSA COM JUSTA CAUSA</t>
+        </is>
+      </c>
       <c r="F289" s="2" t="inlineStr">
         <is>
           <t>ASSISTENTE DE ALIMENTOS E BEBIDAS JUNIOR</t>
@@ -11195,13 +11213,19 @@
       <c r="B299" s="3" t="n">
         <v>46279</v>
       </c>
-      <c r="C299" s="3" t="n"/>
+      <c r="C299" s="3" t="n">
+        <v>46290</v>
+      </c>
       <c r="D299" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E299" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E299" s="2" t="inlineStr">
+        <is>
+          <t>14-PEDIDO ANTES TERMINO CONTRATO</t>
+        </is>
+      </c>
       <c r="F299" s="2" t="inlineStr">
         <is>
           <t>ASSISTENTE DE ALIMENTOS E BEBIDAS JUNIOR</t>
@@ -17743,13 +17767,19 @@
       <c r="B480" s="3" t="n">
         <v>46268</v>
       </c>
-      <c r="C480" s="3" t="n"/>
+      <c r="C480" s="3" t="n">
+        <v>46289</v>
+      </c>
       <c r="D480" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E480" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E480" s="2" t="inlineStr">
+        <is>
+          <t>14-PEDIDO ANTES TERMINO CONTRATO</t>
+        </is>
+      </c>
       <c r="F480" s="2" t="inlineStr">
         <is>
           <t>ASSISTENTE DE ALIMENTOS E BEBIDAS JUNIOR</t>
@@ -17949,13 +17979,19 @@
       <c r="B486" s="3" t="n">
         <v>45589</v>
       </c>
-      <c r="C486" s="3" t="n"/>
+      <c r="C486" s="3" t="n">
+        <v>46293</v>
+      </c>
       <c r="D486" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E486" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E486" s="2" t="inlineStr">
+        <is>
+          <t>06-PEDIDO DE DEMISSÃO</t>
+        </is>
+      </c>
       <c r="F486" s="2" t="inlineStr">
         <is>
           <t>ANALISTA DE RECRUTAMENTO E SELECAO PLENO</t>
@@ -19557,13 +19593,19 @@
       <c r="B530" s="3" t="n">
         <v>45824</v>
       </c>
-      <c r="C530" s="3" t="n"/>
+      <c r="C530" s="3" t="n">
+        <v>46289</v>
+      </c>
       <c r="D530" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E530" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E530" s="2" t="inlineStr">
+        <is>
+          <t>06-PEDIDO DE DEMISSÃO</t>
+        </is>
+      </c>
       <c r="F530" s="2" t="inlineStr">
         <is>
           <t>AUXILIAR DE PRODUCAO</t>
@@ -21937,13 +21979,19 @@
       <c r="B595" s="3" t="n">
         <v>46104</v>
       </c>
-      <c r="C595" s="3" t="n"/>
+      <c r="C595" s="3" t="n">
+        <v>46287</v>
+      </c>
       <c r="D595" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E595" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E595" s="2" t="inlineStr">
+        <is>
+          <t>06-PEDIDO DE DEMISSÃO</t>
+        </is>
+      </c>
       <c r="F595" s="2" t="inlineStr">
         <is>
           <t>ATENDENTE DE SALAO JUNIOR</t>
@@ -27177,13 +27225,19 @@
       <c r="B740" s="3" t="n">
         <v>46209</v>
       </c>
-      <c r="C740" s="3" t="n"/>
+      <c r="C740" s="3" t="n">
+        <v>46288</v>
+      </c>
       <c r="D740" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E740" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E740" s="2" t="inlineStr">
+        <is>
+          <t>04-DISPENSA COM JUSTA CAUSA</t>
+        </is>
+      </c>
       <c r="F740" s="2" t="inlineStr">
         <is>
           <t>ATENDENTE DE SALAO JUNIOR</t>

</xml_diff>

<commit_message>
Base de turnover atualizada automaticamente (30/09/2026 00:31)
</commit_message>
<xml_diff>
--- a/data/dados.xlsx
+++ b/data/dados.xlsx
@@ -602,7 +602,7 @@
       <c r="E4" s="2" t="n"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE SALAO</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>30-CABANA MORUMBI TOWN</t>
+          <t>19-CABANA CAMPO BELO</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE ALIMENTOS E BEBIDAS I</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -1320,7 +1320,7 @@
       <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE SALAO</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1602,7 +1602,7 @@
       <c r="E32" s="2" t="n"/>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE SALAO</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -1612,7 +1612,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>05-CABANA BARRA SHOP</t>
+          <t>23- CABANA BOTAFOGO</t>
         </is>
       </c>
     </row>
@@ -2330,7 +2330,7 @@
       <c r="E52" s="2" t="n"/>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE SALAO</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -2864,7 +2864,7 @@
       <c r="E67" s="2" t="n"/>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE ALIMENTOS E BEBIDAS</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -3792,7 +3792,7 @@
       <c r="E93" s="2" t="n"/>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE ALIMENTOS E BEBIDAS</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -5622,7 +5622,7 @@
       <c r="E144" s="2" t="n"/>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE SALAO</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -6854,7 +6854,7 @@
       <c r="E178" s="2" t="n"/>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE ALIMENTOS E BEBIDAS</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -9828,7 +9828,7 @@
       <c r="E260" s="2" t="n"/>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE SALAO</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -11704,7 +11704,7 @@
       <c r="E312" s="2" t="n"/>
       <c r="F312" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE SALAO</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G312" s="2" t="inlineStr">
@@ -14784,7 +14784,7 @@
       </c>
       <c r="F397" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE SALAO</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G397" s="2" t="inlineStr">
@@ -15558,17 +15558,17 @@
       <c r="E418" s="2" t="n"/>
       <c r="F418" s="2" t="inlineStr">
         <is>
-          <t>ATENDENTE DE SALAO SENIOR</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G418" s="2" t="inlineStr">
         <is>
-          <t>SALÃO</t>
+          <t>LIDERANÇA LOJA</t>
         </is>
       </c>
       <c r="H418" s="2" t="inlineStr">
         <is>
-          <t>05-CABANA BARRA SHOP</t>
+          <t>14-CABANA NITEROI</t>
         </is>
       </c>
     </row>
@@ -16602,7 +16602,7 @@
       <c r="E447" s="2" t="n"/>
       <c r="F447" s="2" t="inlineStr">
         <is>
-          <t>ASSISTENTE DE ALIMENTOS E BEBIDAS SENIOR</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G447" s="2" t="inlineStr">
@@ -17062,7 +17062,7 @@
       <c r="E460" s="2" t="n"/>
       <c r="F460" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE ALIMENTOS E BEBIDAS</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G460" s="2" t="inlineStr">
@@ -20008,17 +20008,17 @@
       <c r="E541" s="2" t="n"/>
       <c r="F541" s="2" t="inlineStr">
         <is>
-          <t>GERENTE DE LOJA</t>
+          <t>COORDENADOR DE OPERAÇÕES</t>
         </is>
       </c>
       <c r="G541" s="2" t="inlineStr">
         <is>
-          <t>LIDERANÇA LOJA</t>
+          <t>OPERAÇÕES LOJAS</t>
         </is>
       </c>
       <c r="H541" s="2" t="inlineStr">
         <is>
-          <t>22-CABANA PINHEIROS</t>
+          <t>01-CABANA MATRIZ</t>
         </is>
       </c>
     </row>
@@ -20840,7 +20840,7 @@
       <c r="E564" s="2" t="n"/>
       <c r="F564" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE ALIMENTOS E BEBIDAS</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G564" s="2" t="inlineStr">
@@ -21512,7 +21512,7 @@
       <c r="E582" s="2" t="n"/>
       <c r="F582" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE ALIMENTOS E BEBIDAS</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G582" s="2" t="inlineStr">
@@ -24648,12 +24648,12 @@
       <c r="E668" s="2" t="n"/>
       <c r="F668" s="2" t="inlineStr">
         <is>
-          <t>ASSISTENTE DE ALIMENTOS E BEBIDAS SENIOR</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G668" s="2" t="inlineStr">
         <is>
-          <t>COZINHA</t>
+          <t>LIDERANÇA LOJA</t>
         </is>
       </c>
       <c r="H668" s="2" t="inlineStr">
@@ -28638,7 +28638,7 @@
       <c r="E779" s="2" t="n"/>
       <c r="F779" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE SALAO</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G779" s="2" t="inlineStr">
@@ -30640,7 +30640,7 @@
       <c r="E834" s="2" t="n"/>
       <c r="F834" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE ALIMENTOS E BEBIDAS</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G834" s="2" t="inlineStr">
@@ -31218,7 +31218,7 @@
       <c r="E850" s="2" t="n"/>
       <c r="F850" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE ALIMENTOS E BEBIDAS</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G850" s="2" t="inlineStr">
@@ -32136,7 +32136,7 @@
       </c>
       <c r="H875" s="2" t="inlineStr">
         <is>
-          <t>14-CABANA NITEROI</t>
+          <t>23- CABANA BOTAFOGO</t>
         </is>
       </c>
     </row>
@@ -36540,12 +36540,12 @@
       <c r="E998" s="2" t="n"/>
       <c r="F998" s="2" t="inlineStr">
         <is>
-          <t>ASSISTENTE DE ALIMENTOS E BEBIDAS SENIOR</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G998" s="2" t="inlineStr">
         <is>
-          <t>COZINHA</t>
+          <t>LIDERANÇA LOJA</t>
         </is>
       </c>
       <c r="H998" s="2" t="inlineStr">
@@ -36872,7 +36872,7 @@
       <c r="E1008" s="2" t="n"/>
       <c r="F1008" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE SALAO</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G1008" s="2" t="inlineStr">
@@ -41838,17 +41838,17 @@
       <c r="E1146" s="2" t="n"/>
       <c r="F1146" s="2" t="inlineStr">
         <is>
-          <t>GERENTE DE LOJA</t>
+          <t>COORDENADOR DE OPERAÇÕES</t>
         </is>
       </c>
       <c r="G1146" s="2" t="inlineStr">
         <is>
-          <t>LIDERANÇA LOJA</t>
+          <t>OPERAÇÕES LOJAS</t>
         </is>
       </c>
       <c r="H1146" s="2" t="inlineStr">
         <is>
-          <t>05-CABANA BARRA SHOP</t>
+          <t>01-CABANA MATRIZ</t>
         </is>
       </c>
     </row>
@@ -44232,7 +44232,7 @@
       <c r="E1212" s="2" t="n"/>
       <c r="F1212" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE ALIMENTOS E BEBIDAS</t>
+          <t>GERENTE DE LOJA</t>
         </is>
       </c>
       <c r="G1212" s="2" t="inlineStr">
@@ -44242,7 +44242,7 @@
       </c>
       <c r="H1212" s="2" t="inlineStr">
         <is>
-          <t>05-CABANA BARRA SHOP</t>
+          <t>14-CABANA NITEROI</t>
         </is>
       </c>
     </row>
@@ -44372,17 +44372,17 @@
       <c r="E1216" s="2" t="n"/>
       <c r="F1216" s="2" t="inlineStr">
         <is>
-          <t>SUPERVISOR DE LOGISTICA</t>
+          <t>CONSULTOR DE B2B</t>
         </is>
       </c>
       <c r="G1216" s="2" t="inlineStr">
         <is>
-          <t>LOGÍSTICA</t>
+          <t>MARKETING</t>
         </is>
       </c>
       <c r="H1216" s="2" t="inlineStr">
         <is>
-          <t>10-CABANA COZINHA CENTRAL</t>
+          <t>01-CABANA MATRIZ</t>
         </is>
       </c>
     </row>
@@ -47046,7 +47046,7 @@
       <c r="E1291" s="2" t="n"/>
       <c r="F1291" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE SALAO</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G1291" s="2" t="inlineStr">
@@ -47302,7 +47302,7 @@
       <c r="E1298" s="2" t="n"/>
       <c r="F1298" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE SALAO</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G1298" s="2" t="inlineStr">
@@ -47312,7 +47312,7 @@
       </c>
       <c r="H1298" s="2" t="inlineStr">
         <is>
-          <t>22-CABANA PINHEIROS</t>
+          <t>02-CABANA LEOPOLDO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Base de turnover atualizada automaticamente (02/10/2026 10:02)
</commit_message>
<xml_diff>
--- a/data/dados.xlsx
+++ b/data/dados.xlsx
@@ -17564,7 +17564,7 @@
       <c r="E474" s="2" t="n"/>
       <c r="F474" s="2" t="inlineStr">
         <is>
-          <t>ASSISTENTE DE ALIMENTOS E BEBIDAS PLENO</t>
+          <t>ASSISTENTE DE ALIMENTOS E BEBIDAS SENIOR</t>
         </is>
       </c>
       <c r="G474" s="2" t="inlineStr">
@@ -26668,7 +26668,7 @@
       <c r="E724" s="2" t="n"/>
       <c r="F724" s="2" t="inlineStr">
         <is>
-          <t>ATENDENTE DE SALAO PLENO</t>
+          <t>ATENDENTE DE SALAO SENIOR</t>
         </is>
       </c>
       <c r="G724" s="2" t="inlineStr">
@@ -43458,7 +43458,7 @@
       <c r="E1191" s="2" t="n"/>
       <c r="F1191" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR (A) DE EXPERIÊNCIA DO CLIENTE</t>
+          <t>LIDER DE EXPERIENCIA DO CONSUMIDOR</t>
         </is>
       </c>
       <c r="G1191" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Base de turnover atualizada automaticamente (08/10/2026 10:01)
</commit_message>
<xml_diff>
--- a/data/dados.xlsx
+++ b/data/dados.xlsx
@@ -2919,13 +2919,19 @@
       <c r="B69" s="3" t="n">
         <v>44410</v>
       </c>
-      <c r="C69" s="3" t="n"/>
+      <c r="C69" s="3" t="n">
+        <v>46196</v>
+      </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>21-DEMISSÃO POR ACORDO MÚTUO AVISO INDENIZADO</t>
+        </is>
+      </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
           <t>COORDENADOR DE LOJA</t>
@@ -3752,7 +3758,7 @@
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>05-CABANA BARRA SHOP</t>
+          <t>23- CABANA BOTAFOGO</t>
         </is>
       </c>
     </row>
@@ -6985,13 +6991,19 @@
       <c r="B182" s="3" t="n">
         <v>44410</v>
       </c>
-      <c r="C182" s="3" t="n"/>
+      <c r="C182" s="3" t="n">
+        <v>46239</v>
+      </c>
       <c r="D182" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E182" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>21-DEMISSÃO POR ACORDO MÚTUO AVISO INDENIZADO</t>
+        </is>
+      </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
           <t>COORDENADOR DE LOJA</t>
@@ -18020,7 +18032,7 @@
       </c>
       <c r="H487" s="2" t="inlineStr">
         <is>
-          <t>14-CABANA NITEROI</t>
+          <t>23- CABANA BOTAFOGO</t>
         </is>
       </c>
     </row>
@@ -39720,7 +39732,7 @@
       <c r="E1088" s="2" t="n"/>
       <c r="F1088" s="2" t="inlineStr">
         <is>
-          <t>COORDENADOR DE SALAO</t>
+          <t>COORDENADOR DE LOJA</t>
         </is>
       </c>
       <c r="G1088" s="2" t="inlineStr">
@@ -41760,7 +41772,7 @@
       </c>
       <c r="H1145" s="2" t="inlineStr">
         <is>
-          <t>02-CABANA LEOPOLDO</t>
+          <t>09-CABANA MOEMA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Base de turnover atualizada automaticamente (11/10/2026 19:54)
</commit_message>
<xml_diff>
--- a/data/dados.xlsx
+++ b/data/dados.xlsx
@@ -11777,13 +11777,19 @@
       <c r="B314" s="3" t="n">
         <v>46268</v>
       </c>
-      <c r="C314" s="3" t="n"/>
+      <c r="C314" s="3" t="n">
+        <v>46300</v>
+      </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E314" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E314" s="2" t="inlineStr">
+        <is>
+          <t>04-DISPENSA COM JUSTA CAUSA</t>
+        </is>
+      </c>
       <c r="F314" s="2" t="inlineStr">
         <is>
           <t>ATENDENTE DE SALAO JUNIOR</t>
@@ -38821,13 +38827,19 @@
       <c r="B1063" s="3" t="n">
         <v>46244</v>
       </c>
-      <c r="C1063" s="3" t="n"/>
+      <c r="C1063" s="3" t="n">
+        <v>46300</v>
+      </c>
       <c r="D1063" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E1063" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E1063" s="2" t="inlineStr">
+        <is>
+          <t>04-DISPENSA COM JUSTA CAUSA</t>
+        </is>
+      </c>
       <c r="F1063" s="2" t="inlineStr">
         <is>
           <t>ASSISTENTE DE ALIMENTOS E BEBIDAS JUNIOR</t>
@@ -48909,13 +48921,19 @@
       <c r="B1344" s="3" t="n">
         <v>46090</v>
       </c>
-      <c r="C1344" s="3" t="n"/>
+      <c r="C1344" s="3" t="n">
+        <v>46300</v>
+      </c>
       <c r="D1344" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E1344" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E1344" s="2" t="inlineStr">
+        <is>
+          <t>04-DISPENSA COM JUSTA CAUSA</t>
+        </is>
+      </c>
       <c r="F1344" s="2" t="inlineStr">
         <is>
           <t>AUXILIAR DE PRODUCAO</t>
@@ -52695,13 +52713,19 @@
       <c r="B1448" s="3" t="n">
         <v>46286</v>
       </c>
-      <c r="C1448" s="3" t="n"/>
+      <c r="C1448" s="3" t="n">
+        <v>46300</v>
+      </c>
       <c r="D1448" s="4" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E1448" s="2" t="n"/>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E1448" s="2" t="inlineStr">
+        <is>
+          <t>14-PEDIDO ANTES TERMINO CONTRATO</t>
+        </is>
+      </c>
       <c r="F1448" s="2" t="inlineStr">
         <is>
           <t>ATENDENTE DE SALAO JUNIOR</t>

</xml_diff>